<commit_message>
Update sea PDHES candidates with new calculated metrics (100 MW, 700 MWh, accurate heads and CAPEX)
</commit_message>
<xml_diff>
--- a/docs/pdhes_adayları_excel/PDHES_Aday_Verileri_Koordinatli_Dinamik_Hesap.xlsx
+++ b/docs/pdhes_adayları_excel/PDHES_Aday_Verileri_Koordinatli_Dinamik_Hesap.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\yazilim_projeler\zPompaj_DHES\docs\pdhes_adayları_excel\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{DC1185E4-8AE7-4FA7-BA1B-5DAC5A360865}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{2E68A87D-4C47-43F3-8990-FA74AE29118C}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="22932" yWindow="-48" windowWidth="23256" windowHeight="12720" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12720" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Aday_Verileri" sheetId="1" r:id="rId1"/>
@@ -460,9 +460,6 @@
     <t>Akdeniz / Taşucu kıyısı</t>
   </si>
   <si>
-    <t>Tuzlu su korozyonu, kıyı izinleri, deniz ekolojisi, uzun su yolu</t>
-  </si>
-  <si>
     <t>https://earth.google.com/web/search/36.230000,33.800000</t>
   </si>
   <si>
@@ -481,9 +478,6 @@
     <t>Akdeniz / Anamur-Bozyazı kıyısı</t>
   </si>
   <si>
-    <t>Çok yüksek düşü; boru hattı, erişim yolu, kıyı/orman izinleri ve korozyon riski</t>
-  </si>
-  <si>
     <t>https://earth.google.com/web/search/36.097000,32.980000</t>
   </si>
   <si>
@@ -499,9 +493,6 @@
     <t>Ege Denizi / Karaburun kıyısı</t>
   </si>
   <si>
-    <t>Kıyı ve doğal sit/orman izinleri; görsel etki, deniz ekolojisi ve korozyon</t>
-  </si>
-  <si>
     <t>https://earth.google.com/web/search/38.629000,26.570000</t>
   </si>
   <si>
@@ -866,6 +857,15 @@
   </si>
   <si>
     <t>Açık Çevrim PDHES</t>
+  </si>
+  <si>
+    <t>Deniz suyu korozyonu, kıyı izinleri, deniz ekolojisi, karst ve sızdırmazlık riski</t>
+  </si>
+  <si>
+    <t>Orta-yüksek düşü; kıyı/orman izinleri, heyelan, korozyon ve sızdırmazlık riski</t>
+  </si>
+  <si>
+    <t>Çok yüksek düşü; doğal sit/orman izinleri, görsel etki, deniz ekolojisi ve yüksek basınçlı su yolu riski</t>
   </si>
 </sst>
 </file>
@@ -980,16 +980,16 @@
     <xf numFmtId="0" fontId="3" fillId="4" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="0" xfId="1" applyAlignment="1">
+      <alignment wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="2" fillId="3" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="left" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="5" fillId="0" borderId="0" xfId="1" applyAlignment="1">
-      <alignment wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="1"/>
   </cellXfs>
   <cellStyles count="2">
     <cellStyle name="Köprü" xfId="1" builtinId="8"/>
@@ -1430,8 +1430,8 @@
       <c r="B2" t="s">
         <v>44</v>
       </c>
-      <c r="C2" s="13" t="s">
-        <v>275</v>
+      <c r="C2" s="11" t="s">
+        <v>272</v>
       </c>
       <c r="D2" t="s">
         <v>45</v>
@@ -1588,8 +1588,8 @@
       <c r="B3" t="s">
         <v>54</v>
       </c>
-      <c r="C3" s="13" t="s">
-        <v>275</v>
+      <c r="C3" s="11" t="s">
+        <v>272</v>
       </c>
       <c r="D3" t="s">
         <v>55</v>
@@ -1746,8 +1746,8 @@
       <c r="B4" t="s">
         <v>63</v>
       </c>
-      <c r="C4" s="13" t="s">
-        <v>275</v>
+      <c r="C4" s="11" t="s">
+        <v>272</v>
       </c>
       <c r="D4" t="s">
         <v>64</v>
@@ -1904,8 +1904,8 @@
       <c r="B5" t="s">
         <v>71</v>
       </c>
-      <c r="C5" s="13" t="s">
-        <v>275</v>
+      <c r="C5" s="11" t="s">
+        <v>272</v>
       </c>
       <c r="D5" t="s">
         <v>72</v>
@@ -2062,8 +2062,8 @@
       <c r="B6" t="s">
         <v>79</v>
       </c>
-      <c r="C6" s="13" t="s">
-        <v>275</v>
+      <c r="C6" s="11" t="s">
+        <v>272</v>
       </c>
       <c r="D6" t="s">
         <v>64</v>
@@ -2220,8 +2220,8 @@
       <c r="B7" t="s">
         <v>85</v>
       </c>
-      <c r="C7" s="13" t="s">
-        <v>275</v>
+      <c r="C7" s="11" t="s">
+        <v>272</v>
       </c>
       <c r="D7" t="s">
         <v>86</v>
@@ -2378,8 +2378,8 @@
       <c r="B8" t="s">
         <v>92</v>
       </c>
-      <c r="C8" s="13" t="s">
-        <v>275</v>
+      <c r="C8" s="11" t="s">
+        <v>272</v>
       </c>
       <c r="D8" t="s">
         <v>55</v>
@@ -2536,8 +2536,8 @@
       <c r="B9" t="s">
         <v>98</v>
       </c>
-      <c r="C9" s="13" t="s">
-        <v>275</v>
+      <c r="C9" s="11" t="s">
+        <v>272</v>
       </c>
       <c r="D9" t="s">
         <v>99</v>
@@ -2694,8 +2694,8 @@
       <c r="B10" t="s">
         <v>106</v>
       </c>
-      <c r="C10" s="13" t="s">
-        <v>275</v>
+      <c r="C10" s="11" t="s">
+        <v>272</v>
       </c>
       <c r="D10" t="s">
         <v>107</v>
@@ -2852,8 +2852,8 @@
       <c r="B11" t="s">
         <v>113</v>
       </c>
-      <c r="C11" s="13" t="s">
-        <v>275</v>
+      <c r="C11" s="11" t="s">
+        <v>272</v>
       </c>
       <c r="D11" t="s">
         <v>114</v>
@@ -3010,8 +3010,8 @@
       <c r="B12" t="s">
         <v>121</v>
       </c>
-      <c r="C12" s="13" t="s">
-        <v>275</v>
+      <c r="C12" s="11" t="s">
+        <v>272</v>
       </c>
       <c r="D12" t="s">
         <v>122</v>
@@ -3168,8 +3168,8 @@
       <c r="B13" t="s">
         <v>128</v>
       </c>
-      <c r="C13" s="13" t="s">
-        <v>275</v>
+      <c r="C13" s="11" t="s">
+        <v>272</v>
       </c>
       <c r="D13" t="s">
         <v>129</v>
@@ -3361,15 +3361,13 @@
         <v>33.844000000000001</v>
       </c>
       <c r="N14" s="4">
-        <f t="shared" si="1"/>
-        <v>780</v>
+        <v>500</v>
       </c>
       <c r="O14" s="4">
-        <v>780</v>
+        <v>500</v>
       </c>
       <c r="P14" s="4">
-        <f t="shared" si="2"/>
-        <v>756.6</v>
+        <v>485</v>
       </c>
       <c r="Q14" s="4">
         <f>Input_Parametreleri!$B$7</f>
@@ -3377,11 +3375,11 @@
       </c>
       <c r="R14" s="4">
         <f>IFERROR(E14*1000000/(Input_Parametreleri!$B$2*Input_Parametreleri!$B$3*P14*Input_Parametreleri!$B$4),0)</f>
-        <v>14.970011922416894</v>
+        <v>23.353218598970358</v>
       </c>
       <c r="S14" s="4">
         <f>IFERROR(G14*3600000000/(Input_Parametreleri!$B$2*Input_Parametreleri!$B$3*P14*Input_Parametreleri!$B$4)/1000000,0)</f>
-        <v>0.37724430044490576</v>
+        <v>0.58850110869405303</v>
       </c>
       <c r="T14" s="6">
         <f>Input_Parametreleri!$B$6</f>
@@ -3436,45 +3434,40 @@
         <v>18.484615384615385</v>
       </c>
       <c r="AG14" s="4">
-        <f>Input_Parametreleri!$B$13*(1+IF(P14&lt;200,Input_Parametreleri!$B$17,0)+IF(O14&gt;700,Input_Parametreleri!$B$16,0)+IF(ISNUMBER(SEARCH("Deniz",C14)),Input_Parametreleri!$B$15-1,0))</f>
-        <v>2244</v>
+        <v>1670.7716329078846</v>
       </c>
       <c r="AH14" s="4">
-        <f t="shared" si="8"/>
-        <v>224.4</v>
+        <v>167.07716329078846</v>
       </c>
       <c r="AI14" s="4">
-        <f>AH14*Input_Parametreleri!$B$14</f>
-        <v>3.3660000000000001</v>
+        <v>2.5061574493618268</v>
       </c>
       <c r="AJ14" s="4">
-        <f t="shared" si="9"/>
-        <v>15.118615384615385</v>
+        <v>15.978457935253559</v>
       </c>
       <c r="AK14" s="4">
-        <f t="shared" si="10"/>
-        <v>14.842629056384895</v>
+        <v>10.456400984863697</v>
       </c>
       <c r="AL14" t="s">
         <v>47</v>
       </c>
       <c r="AM14" t="s">
-        <v>140</v>
+        <v>273</v>
       </c>
       <c r="AN14" t="s">
         <v>49</v>
       </c>
       <c r="AO14" t="s">
+        <v>140</v>
+      </c>
+      <c r="AP14" t="s">
         <v>141</v>
       </c>
-      <c r="AP14" t="s">
+      <c r="AQ14" t="s">
         <v>142</v>
       </c>
-      <c r="AQ14" t="s">
+      <c r="AR14" t="s">
         <v>143</v>
-      </c>
-      <c r="AR14" t="s">
-        <v>144</v>
       </c>
     </row>
     <row r="15" spans="1:44" x14ac:dyDescent="0.3">
@@ -3482,7 +3475,7 @@
         <v>14</v>
       </c>
       <c r="B15" t="s">
-        <v>145</v>
+        <v>144</v>
       </c>
       <c r="C15" t="s">
         <v>137</v>
@@ -3501,7 +3494,7 @@
         <v>700</v>
       </c>
       <c r="H15" t="s">
-        <v>146</v>
+        <v>145</v>
       </c>
       <c r="I15" s="5">
         <v>36.097000000000001</v>
@@ -3519,15 +3512,13 @@
         <v>33.020000000000003</v>
       </c>
       <c r="N15" s="4">
-        <f t="shared" si="1"/>
-        <v>900</v>
+        <v>600</v>
       </c>
       <c r="O15" s="4">
-        <v>900</v>
+        <v>600</v>
       </c>
       <c r="P15" s="4">
-        <f t="shared" si="2"/>
-        <v>873</v>
+        <v>582</v>
       </c>
       <c r="Q15" s="4">
         <f>Input_Parametreleri!$B$7</f>
@@ -3535,11 +3526,11 @@
       </c>
       <c r="R15" s="4">
         <f>IFERROR(E15*1000000/(Input_Parametreleri!$B$2*Input_Parametreleri!$B$3*P15*Input_Parametreleri!$B$4),0)</f>
-        <v>12.97401033276131</v>
+        <v>19.461015499141965</v>
       </c>
       <c r="S15" s="4">
         <f>IFERROR(G15*3600000000/(Input_Parametreleri!$B$2*Input_Parametreleri!$B$3*P15*Input_Parametreleri!$B$4)/1000000,0)</f>
-        <v>0.32694506038558502</v>
+        <v>0.49041759057837747</v>
       </c>
       <c r="T15" s="6">
         <f>Input_Parametreleri!$B$6</f>
@@ -3594,45 +3585,40 @@
         <v>18.484615384615385</v>
       </c>
       <c r="AG15" s="4">
-        <f>Input_Parametreleri!$B$13*(1+IF(P15&lt;200,Input_Parametreleri!$B$17,0)+IF(O15&gt;700,Input_Parametreleri!$B$16,0)+IF(ISNUMBER(SEARCH("Deniz",C15)),Input_Parametreleri!$B$15-1,0))</f>
-        <v>2244</v>
+        <v>1672.7452263636155</v>
       </c>
       <c r="AH15" s="4">
-        <f t="shared" si="8"/>
-        <v>224.4</v>
+        <v>167.27452263636155</v>
       </c>
       <c r="AI15" s="4">
-        <f>AH15*Input_Parametreleri!$B$14</f>
-        <v>3.3660000000000001</v>
+        <v>2.5091178395454232</v>
       </c>
       <c r="AJ15" s="4">
-        <f t="shared" si="9"/>
-        <v>15.118615384615385</v>
+        <v>15.975497545069961</v>
       </c>
       <c r="AK15" s="4">
-        <f t="shared" si="10"/>
-        <v>14.842629056384895</v>
+        <v>10.470692519243789</v>
       </c>
       <c r="AL15" t="s">
         <v>47</v>
       </c>
       <c r="AM15" t="s">
-        <v>147</v>
+        <v>274</v>
       </c>
       <c r="AN15" t="s">
         <v>49</v>
       </c>
       <c r="AO15" t="s">
-        <v>148</v>
+        <v>146</v>
       </c>
       <c r="AP15" t="s">
-        <v>149</v>
+        <v>147</v>
       </c>
       <c r="AQ15" t="s">
+        <v>142</v>
+      </c>
+      <c r="AR15" t="s">
         <v>143</v>
-      </c>
-      <c r="AR15" t="s">
-        <v>144</v>
       </c>
     </row>
     <row r="16" spans="1:44" x14ac:dyDescent="0.3">
@@ -3640,13 +3626,13 @@
         <v>15</v>
       </c>
       <c r="B16" t="s">
-        <v>150</v>
+        <v>148</v>
       </c>
       <c r="C16" t="s">
         <v>137</v>
       </c>
       <c r="D16" t="s">
-        <v>151</v>
+        <v>149</v>
       </c>
       <c r="E16" s="4">
         <v>100</v>
@@ -3659,7 +3645,7 @@
         <v>700</v>
       </c>
       <c r="H16" t="s">
-        <v>152</v>
+        <v>150</v>
       </c>
       <c r="I16" s="5">
         <v>38.628999999999998</v>
@@ -3677,15 +3663,13 @@
         <v>26.61</v>
       </c>
       <c r="N16" s="4">
-        <f t="shared" si="1"/>
-        <v>620</v>
+        <v>900</v>
       </c>
       <c r="O16" s="4">
-        <v>620</v>
+        <v>900</v>
       </c>
       <c r="P16" s="4">
-        <f t="shared" si="2"/>
-        <v>601.4</v>
+        <v>873</v>
       </c>
       <c r="Q16" s="4">
         <f>Input_Parametreleri!$B$7</f>
@@ -3693,11 +3677,11 @@
       </c>
       <c r="R16" s="4">
         <f>IFERROR(E16*1000000/(Input_Parametreleri!$B$2*Input_Parametreleri!$B$3*P16*Input_Parametreleri!$B$4),0)</f>
-        <v>18.833240805621255</v>
+        <v>12.97401033276131</v>
       </c>
       <c r="S16" s="4">
         <f>IFERROR(G16*3600000000/(Input_Parametreleri!$B$2*Input_Parametreleri!$B$3*P16*Input_Parametreleri!$B$4)/1000000,0)</f>
-        <v>0.47459766830165556</v>
+        <v>0.32694506038558502</v>
       </c>
       <c r="T16" s="6">
         <f>Input_Parametreleri!$B$6</f>
@@ -3752,45 +3736,40 @@
         <v>18.484615384615385</v>
       </c>
       <c r="AG16" s="4">
-        <f>Input_Parametreleri!$B$13*(1+IF(P16&lt;200,Input_Parametreleri!$B$17,0)+IF(O16&gt;700,Input_Parametreleri!$B$16,0)+IF(ISNUMBER(SEARCH("Deniz",C16)),Input_Parametreleri!$B$15-1,0))</f>
-        <v>2040</v>
+        <v>2107.9561305702664</v>
       </c>
       <c r="AH16" s="4">
-        <f t="shared" si="8"/>
-        <v>204</v>
+        <v>210.79561305702663</v>
       </c>
       <c r="AI16" s="4">
-        <f>AH16*Input_Parametreleri!$B$14</f>
-        <v>3.06</v>
+        <v>3.1619341958553995</v>
       </c>
       <c r="AJ16" s="4">
-        <f t="shared" si="9"/>
-        <v>15.424615384615384</v>
+        <v>15.322681188759985</v>
       </c>
       <c r="AK16" s="4">
-        <f t="shared" si="10"/>
-        <v>13.225613405146619</v>
+        <v>13.757097107238426</v>
       </c>
       <c r="AL16" t="s">
         <v>47</v>
       </c>
       <c r="AM16" t="s">
-        <v>153</v>
+        <v>275</v>
       </c>
       <c r="AN16" t="s">
         <v>49</v>
       </c>
       <c r="AO16" t="s">
-        <v>154</v>
+        <v>151</v>
       </c>
       <c r="AP16" t="s">
-        <v>155</v>
+        <v>152</v>
       </c>
       <c r="AQ16" t="s">
+        <v>142</v>
+      </c>
+      <c r="AR16" t="s">
         <v>143</v>
-      </c>
-      <c r="AR16" t="s">
-        <v>144</v>
       </c>
     </row>
   </sheetData>
@@ -3872,7 +3851,7 @@
         <v>1</v>
       </c>
       <c r="C1" s="1" t="s">
-        <v>156</v>
+        <v>153</v>
       </c>
       <c r="D1" s="1" t="s">
         <v>8</v>
@@ -3881,7 +3860,7 @@
         <v>9</v>
       </c>
       <c r="F1" s="1" t="s">
-        <v>157</v>
+        <v>154</v>
       </c>
       <c r="G1" s="1" t="s">
         <v>11</v>
@@ -3890,7 +3869,7 @@
         <v>12</v>
       </c>
       <c r="I1" s="1" t="s">
-        <v>158</v>
+        <v>155</v>
       </c>
       <c r="J1" s="1" t="s">
         <v>14</v>
@@ -3899,10 +3878,10 @@
         <v>15</v>
       </c>
       <c r="L1" s="1" t="s">
-        <v>159</v>
+        <v>156</v>
       </c>
       <c r="M1" s="1" t="s">
-        <v>160</v>
+        <v>157</v>
       </c>
       <c r="N1" s="1" t="s">
         <v>40</v>
@@ -3911,13 +3890,13 @@
         <v>41</v>
       </c>
       <c r="P1" s="1" t="s">
-        <v>161</v>
+        <v>158</v>
       </c>
       <c r="Q1" s="1" t="s">
-        <v>162</v>
+        <v>159</v>
       </c>
       <c r="R1" s="1" t="s">
-        <v>163</v>
+        <v>160</v>
       </c>
     </row>
     <row r="2" spans="1:18" ht="28.8" x14ac:dyDescent="0.3">
@@ -3961,10 +3940,10 @@
       <c r="M2" s="3">
         <v>4.0510000000000002</v>
       </c>
-      <c r="N2" s="12" t="s">
+      <c r="N2" s="10" t="s">
         <v>50</v>
       </c>
-      <c r="O2" s="12" t="s">
+      <c r="O2" s="10" t="s">
         <v>51</v>
       </c>
       <c r="P2" s="2" t="s">
@@ -3974,7 +3953,7 @@
         <v>53</v>
       </c>
       <c r="R2" s="2" t="s">
-        <v>164</v>
+        <v>161</v>
       </c>
     </row>
     <row r="3" spans="1:18" ht="28.8" x14ac:dyDescent="0.3">
@@ -4021,7 +4000,7 @@
       <c r="N3" s="2" t="s">
         <v>59</v>
       </c>
-      <c r="O3" s="12" t="s">
+      <c r="O3" s="10" t="s">
         <v>60</v>
       </c>
       <c r="P3" s="2" t="s">
@@ -4031,7 +4010,7 @@
         <v>62</v>
       </c>
       <c r="R3" s="2" t="s">
-        <v>164</v>
+        <v>161</v>
       </c>
     </row>
     <row r="4" spans="1:18" ht="28.8" x14ac:dyDescent="0.3">
@@ -4088,7 +4067,7 @@
         <v>70</v>
       </c>
       <c r="R4" s="2" t="s">
-        <v>164</v>
+        <v>161</v>
       </c>
     </row>
     <row r="5" spans="1:18" ht="28.8" x14ac:dyDescent="0.3">
@@ -4145,7 +4124,7 @@
         <v>78</v>
       </c>
       <c r="R5" s="2" t="s">
-        <v>164</v>
+        <v>161</v>
       </c>
     </row>
     <row r="6" spans="1:18" ht="28.8" x14ac:dyDescent="0.3">
@@ -4202,7 +4181,7 @@
         <v>62</v>
       </c>
       <c r="R6" s="2" t="s">
-        <v>164</v>
+        <v>161</v>
       </c>
     </row>
     <row r="7" spans="1:18" ht="28.8" x14ac:dyDescent="0.3">
@@ -4259,7 +4238,7 @@
         <v>62</v>
       </c>
       <c r="R7" s="2" t="s">
-        <v>164</v>
+        <v>161</v>
       </c>
     </row>
     <row r="8" spans="1:18" ht="28.8" x14ac:dyDescent="0.3">
@@ -4316,7 +4295,7 @@
         <v>62</v>
       </c>
       <c r="R8" s="2" t="s">
-        <v>164</v>
+        <v>161</v>
       </c>
     </row>
     <row r="9" spans="1:18" ht="28.8" x14ac:dyDescent="0.3">
@@ -4373,7 +4352,7 @@
         <v>105</v>
       </c>
       <c r="R9" s="2" t="s">
-        <v>164</v>
+        <v>161</v>
       </c>
     </row>
     <row r="10" spans="1:18" ht="28.8" x14ac:dyDescent="0.3">
@@ -4430,7 +4409,7 @@
         <v>62</v>
       </c>
       <c r="R10" s="2" t="s">
-        <v>164</v>
+        <v>161</v>
       </c>
     </row>
     <row r="11" spans="1:18" ht="43.2" x14ac:dyDescent="0.3">
@@ -4487,7 +4466,7 @@
         <v>120</v>
       </c>
       <c r="R11" s="2" t="s">
-        <v>164</v>
+        <v>161</v>
       </c>
     </row>
     <row r="12" spans="1:18" ht="28.8" x14ac:dyDescent="0.3">
@@ -4544,7 +4523,7 @@
         <v>62</v>
       </c>
       <c r="R12" s="2" t="s">
-        <v>164</v>
+        <v>161</v>
       </c>
     </row>
     <row r="13" spans="1:18" ht="28.8" x14ac:dyDescent="0.3">
@@ -4601,7 +4580,7 @@
         <v>135</v>
       </c>
       <c r="R13" s="2" t="s">
-        <v>164</v>
+        <v>161</v>
       </c>
     </row>
     <row r="14" spans="1:18" ht="28.8" x14ac:dyDescent="0.3">
@@ -4646,19 +4625,19 @@
         <v>6.5</v>
       </c>
       <c r="N14" s="2" t="s">
+        <v>140</v>
+      </c>
+      <c r="O14" s="2" t="s">
         <v>141</v>
       </c>
-      <c r="O14" s="2" t="s">
+      <c r="P14" s="2" t="s">
         <v>142</v>
       </c>
-      <c r="P14" s="2" t="s">
+      <c r="Q14" s="2" t="s">
         <v>143</v>
       </c>
-      <c r="Q14" s="2" t="s">
-        <v>144</v>
-      </c>
       <c r="R14" s="2" t="s">
-        <v>164</v>
+        <v>161</v>
       </c>
     </row>
     <row r="15" spans="1:18" ht="28.8" x14ac:dyDescent="0.3">
@@ -4666,10 +4645,10 @@
         <v>14</v>
       </c>
       <c r="B15" s="2" t="s">
+        <v>144</v>
+      </c>
+      <c r="C15" s="2" t="s">
         <v>145</v>
-      </c>
-      <c r="C15" s="2" t="s">
-        <v>146</v>
       </c>
       <c r="D15" s="7">
         <v>36.097000000000001</v>
@@ -4703,19 +4682,19 @@
         <v>8.5</v>
       </c>
       <c r="N15" s="2" t="s">
-        <v>148</v>
+        <v>146</v>
       </c>
       <c r="O15" s="2" t="s">
-        <v>149</v>
+        <v>147</v>
       </c>
       <c r="P15" s="2" t="s">
+        <v>142</v>
+      </c>
+      <c r="Q15" s="2" t="s">
         <v>143</v>
       </c>
-      <c r="Q15" s="2" t="s">
-        <v>144</v>
-      </c>
       <c r="R15" s="2" t="s">
-        <v>164</v>
+        <v>161</v>
       </c>
     </row>
     <row r="16" spans="1:18" ht="28.8" x14ac:dyDescent="0.3">
@@ -4723,10 +4702,10 @@
         <v>15</v>
       </c>
       <c r="B16" s="2" t="s">
+        <v>148</v>
+      </c>
+      <c r="C16" s="2" t="s">
         <v>150</v>
-      </c>
-      <c r="C16" s="2" t="s">
-        <v>152</v>
       </c>
       <c r="D16" s="7">
         <v>38.628999999999998</v>
@@ -4760,19 +4739,19 @@
         <v>5</v>
       </c>
       <c r="N16" s="2" t="s">
-        <v>154</v>
+        <v>151</v>
       </c>
       <c r="O16" s="2" t="s">
-        <v>155</v>
+        <v>152</v>
       </c>
       <c r="P16" s="2" t="s">
+        <v>142</v>
+      </c>
+      <c r="Q16" s="2" t="s">
         <v>143</v>
       </c>
-      <c r="Q16" s="2" t="s">
-        <v>144</v>
-      </c>
       <c r="R16" s="2" t="s">
-        <v>164</v>
+        <v>161</v>
       </c>
     </row>
   </sheetData>
@@ -4800,240 +4779,240 @@
   <sheetData>
     <row r="1" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A1" s="1" t="s">
+        <v>162</v>
+      </c>
+      <c r="B1" s="1" t="s">
+        <v>163</v>
+      </c>
+      <c r="C1" s="1" t="s">
+        <v>164</v>
+      </c>
+      <c r="D1" s="1" t="s">
         <v>165</v>
-      </c>
-      <c r="B1" s="1" t="s">
-        <v>166</v>
-      </c>
-      <c r="C1" s="1" t="s">
-        <v>167</v>
-      </c>
-      <c r="D1" s="1" t="s">
-        <v>168</v>
       </c>
     </row>
     <row r="2" spans="1:4" ht="28.8" x14ac:dyDescent="0.3">
       <c r="A2" s="2" t="s">
-        <v>169</v>
+        <v>166</v>
       </c>
       <c r="B2" s="3">
         <v>1000</v>
       </c>
       <c r="C2" s="2" t="s">
-        <v>170</v>
+        <v>167</v>
       </c>
       <c r="D2" s="2" t="s">
-        <v>171</v>
+        <v>168</v>
       </c>
     </row>
     <row r="3" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A3" s="2" t="s">
-        <v>172</v>
+        <v>169</v>
       </c>
       <c r="B3" s="3">
         <v>9.81</v>
       </c>
       <c r="C3" s="2" t="s">
-        <v>173</v>
+        <v>170</v>
       </c>
       <c r="D3" s="2" t="s">
-        <v>174</v>
+        <v>171</v>
       </c>
     </row>
     <row r="4" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A4" s="2" t="s">
-        <v>175</v>
+        <v>172</v>
       </c>
       <c r="B4" s="3">
         <v>0.9</v>
       </c>
       <c r="C4" s="2" t="s">
-        <v>176</v>
+        <v>173</v>
       </c>
       <c r="D4" s="2" t="s">
-        <v>177</v>
+        <v>174</v>
       </c>
     </row>
     <row r="5" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A5" s="2" t="s">
-        <v>178</v>
+        <v>175</v>
       </c>
       <c r="B5" s="3">
         <v>0.86</v>
       </c>
       <c r="C5" s="2" t="s">
+        <v>173</v>
+      </c>
+      <c r="D5" s="2" t="s">
         <v>176</v>
-      </c>
-      <c r="D5" s="2" t="s">
-        <v>179</v>
       </c>
     </row>
     <row r="6" spans="1:4" ht="28.8" x14ac:dyDescent="0.3">
       <c r="A6" s="2" t="s">
-        <v>180</v>
+        <v>177</v>
       </c>
       <c r="B6" s="3">
         <v>0.78</v>
       </c>
       <c r="C6" s="2" t="s">
-        <v>176</v>
+        <v>173</v>
       </c>
       <c r="D6" s="2" t="s">
-        <v>181</v>
+        <v>178</v>
       </c>
     </row>
     <row r="7" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A7" s="2" t="s">
-        <v>182</v>
+        <v>179</v>
       </c>
       <c r="B7" s="3">
         <v>0.03</v>
       </c>
       <c r="C7" s="2" t="s">
-        <v>176</v>
+        <v>173</v>
       </c>
       <c r="D7" s="2" t="s">
-        <v>183</v>
+        <v>180</v>
       </c>
     </row>
     <row r="8" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A8" s="2" t="s">
-        <v>184</v>
+        <v>181</v>
       </c>
       <c r="B8" s="3">
         <v>300</v>
       </c>
       <c r="C8" s="2" t="s">
-        <v>185</v>
+        <v>182</v>
       </c>
       <c r="D8" s="2" t="s">
-        <v>186</v>
+        <v>183</v>
       </c>
     </row>
     <row r="9" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A9" s="2" t="s">
-        <v>187</v>
+        <v>184</v>
       </c>
       <c r="B9" s="3">
         <v>110</v>
       </c>
       <c r="C9" s="2" t="s">
-        <v>188</v>
+        <v>185</v>
       </c>
       <c r="D9" s="2" t="s">
-        <v>189</v>
+        <v>186</v>
       </c>
     </row>
     <row r="10" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A10" s="2" t="s">
-        <v>190</v>
+        <v>187</v>
       </c>
       <c r="B10" s="3">
         <v>45</v>
       </c>
       <c r="C10" s="2" t="s">
+        <v>185</v>
+      </c>
+      <c r="D10" s="2" t="s">
         <v>188</v>
-      </c>
-      <c r="D10" s="2" t="s">
-        <v>191</v>
       </c>
     </row>
     <row r="11" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A11" s="2" t="s">
-        <v>192</v>
+        <v>189</v>
       </c>
       <c r="B11" s="3">
         <v>45000</v>
       </c>
       <c r="C11" s="2" t="s">
-        <v>193</v>
+        <v>190</v>
       </c>
       <c r="D11" s="2" t="s">
-        <v>194</v>
+        <v>191</v>
       </c>
     </row>
     <row r="12" spans="1:4" ht="28.8" x14ac:dyDescent="0.3">
       <c r="A12" s="2" t="s">
-        <v>195</v>
+        <v>192</v>
       </c>
       <c r="B12" s="3">
         <v>30000</v>
       </c>
       <c r="C12" s="2" t="s">
+        <v>190</v>
+      </c>
+      <c r="D12" s="2" t="s">
         <v>193</v>
-      </c>
-      <c r="D12" s="2" t="s">
-        <v>196</v>
       </c>
     </row>
     <row r="13" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A13" s="2" t="s">
-        <v>197</v>
+        <v>194</v>
       </c>
       <c r="B13" s="3">
         <v>1700</v>
       </c>
       <c r="C13" s="2" t="s">
-        <v>198</v>
+        <v>195</v>
       </c>
       <c r="D13" s="2" t="s">
-        <v>199</v>
+        <v>196</v>
       </c>
     </row>
     <row r="14" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A14" s="2" t="s">
-        <v>200</v>
+        <v>197</v>
       </c>
       <c r="B14" s="3">
         <v>1.4999999999999999E-2</v>
       </c>
       <c r="C14" s="2" t="s">
-        <v>201</v>
+        <v>198</v>
       </c>
       <c r="D14" s="2" t="s">
-        <v>202</v>
+        <v>199</v>
       </c>
     </row>
     <row r="15" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A15" s="2" t="s">
-        <v>203</v>
+        <v>200</v>
       </c>
       <c r="B15" s="3">
         <v>1.2</v>
       </c>
       <c r="C15" s="2" t="s">
-        <v>204</v>
+        <v>201</v>
       </c>
       <c r="D15" s="2" t="s">
-        <v>205</v>
+        <v>202</v>
       </c>
     </row>
     <row r="16" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A16" s="2" t="s">
-        <v>206</v>
+        <v>203</v>
       </c>
       <c r="B16" s="3">
         <v>0.12</v>
       </c>
       <c r="C16" s="2" t="s">
-        <v>207</v>
+        <v>204</v>
       </c>
       <c r="D16" s="2" t="s">
-        <v>208</v>
+        <v>205</v>
       </c>
     </row>
     <row r="17" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A17" s="2" t="s">
-        <v>209</v>
+        <v>206</v>
       </c>
       <c r="B17" s="3">
         <v>0.1</v>
       </c>
       <c r="C17" s="2" t="s">
+        <v>204</v>
+      </c>
+      <c r="D17" s="2" t="s">
         <v>207</v>
-      </c>
-      <c r="D17" s="2" t="s">
-        <v>210</v>
       </c>
     </row>
   </sheetData>
@@ -5052,99 +5031,99 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:4" ht="15" x14ac:dyDescent="0.35">
-      <c r="A1" s="10" t="s">
-        <v>211</v>
-      </c>
-      <c r="B1" s="11"/>
-      <c r="C1" s="11"/>
-      <c r="D1" s="11"/>
+      <c r="A1" s="12" t="s">
+        <v>208</v>
+      </c>
+      <c r="B1" s="13"/>
+      <c r="C1" s="13"/>
+      <c r="D1" s="13"/>
     </row>
     <row r="2" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A2" s="9" t="s">
-        <v>212</v>
+        <v>209</v>
       </c>
       <c r="B2" t="s">
-        <v>213</v>
+        <v>210</v>
       </c>
     </row>
     <row r="3" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A3" s="9" t="s">
-        <v>214</v>
+        <v>211</v>
       </c>
       <c r="B3" t="s">
-        <v>215</v>
+        <v>212</v>
       </c>
     </row>
     <row r="4" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A4" s="9" t="s">
-        <v>216</v>
+        <v>213</v>
       </c>
       <c r="B4" t="s">
-        <v>217</v>
+        <v>214</v>
       </c>
     </row>
     <row r="5" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A5" s="9" t="s">
-        <v>218</v>
+        <v>215</v>
       </c>
       <c r="B5" t="s">
-        <v>219</v>
+        <v>216</v>
       </c>
     </row>
     <row r="6" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A6" s="9" t="s">
-        <v>220</v>
+        <v>217</v>
       </c>
       <c r="B6" t="s">
-        <v>221</v>
+        <v>218</v>
       </c>
     </row>
     <row r="7" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A7" s="9" t="s">
-        <v>222</v>
+        <v>219</v>
       </c>
       <c r="B7" t="s">
-        <v>223</v>
+        <v>220</v>
       </c>
     </row>
     <row r="8" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A8" s="9" t="s">
-        <v>224</v>
+        <v>221</v>
       </c>
       <c r="B8" t="s">
-        <v>225</v>
+        <v>222</v>
       </c>
     </row>
     <row r="9" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A9" s="9" t="s">
-        <v>226</v>
+        <v>223</v>
       </c>
       <c r="B9" t="s">
-        <v>227</v>
+        <v>224</v>
       </c>
     </row>
     <row r="10" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A10" s="9" t="s">
-        <v>228</v>
+        <v>225</v>
       </c>
       <c r="B10" t="s">
-        <v>229</v>
+        <v>226</v>
       </c>
     </row>
     <row r="11" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A11" s="9" t="s">
-        <v>230</v>
+        <v>227</v>
       </c>
       <c r="B11" t="s">
-        <v>231</v>
+        <v>228</v>
       </c>
     </row>
     <row r="12" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A12" s="9" t="s">
-        <v>232</v>
+        <v>229</v>
       </c>
       <c r="B12" t="s">
-        <v>233</v>
+        <v>230</v>
       </c>
     </row>
   </sheetData>
@@ -5173,25 +5152,25 @@
         <v>1</v>
       </c>
       <c r="C1" s="8" t="s">
+        <v>231</v>
+      </c>
+      <c r="D1" s="8" t="s">
+        <v>232</v>
+      </c>
+      <c r="E1" s="8" t="s">
+        <v>233</v>
+      </c>
+      <c r="F1" s="8" t="s">
         <v>234</v>
       </c>
-      <c r="D1" s="8" t="s">
+      <c r="G1" s="8" t="s">
         <v>235</v>
       </c>
-      <c r="E1" s="8" t="s">
+      <c r="H1" s="1" t="s">
         <v>236</v>
       </c>
-      <c r="F1" s="8" t="s">
+      <c r="I1" s="1" t="s">
         <v>237</v>
-      </c>
-      <c r="G1" s="8" t="s">
-        <v>238</v>
-      </c>
-      <c r="H1" s="1" t="s">
-        <v>239</v>
-      </c>
-      <c r="I1" s="1" t="s">
-        <v>240</v>
       </c>
     </row>
     <row r="2" spans="1:9" x14ac:dyDescent="0.3">
@@ -5226,7 +5205,7 @@
         <v>C - Koşullu</v>
       </c>
       <c r="I2" t="s">
-        <v>241</v>
+        <v>238</v>
       </c>
     </row>
     <row r="3" spans="1:9" x14ac:dyDescent="0.3">
@@ -5261,7 +5240,7 @@
         <v>C - Koşullu</v>
       </c>
       <c r="I3" t="s">
-        <v>241</v>
+        <v>238</v>
       </c>
     </row>
     <row r="4" spans="1:9" x14ac:dyDescent="0.3">
@@ -5296,7 +5275,7 @@
         <v>B - İncelenmeli</v>
       </c>
       <c r="I4" t="s">
-        <v>241</v>
+        <v>238</v>
       </c>
     </row>
     <row r="5" spans="1:9" x14ac:dyDescent="0.3">
@@ -5331,7 +5310,7 @@
         <v>C - Koşullu</v>
       </c>
       <c r="I5" t="s">
-        <v>241</v>
+        <v>238</v>
       </c>
     </row>
     <row r="6" spans="1:9" x14ac:dyDescent="0.3">
@@ -5366,7 +5345,7 @@
         <v>B - İncelenmeli</v>
       </c>
       <c r="I6" t="s">
-        <v>241</v>
+        <v>238</v>
       </c>
     </row>
     <row r="7" spans="1:9" x14ac:dyDescent="0.3">
@@ -5401,7 +5380,7 @@
         <v>C - Koşullu</v>
       </c>
       <c r="I7" t="s">
-        <v>241</v>
+        <v>238</v>
       </c>
     </row>
     <row r="8" spans="1:9" x14ac:dyDescent="0.3">
@@ -5436,7 +5415,7 @@
         <v>B - İncelenmeli</v>
       </c>
       <c r="I8" t="s">
-        <v>241</v>
+        <v>238</v>
       </c>
     </row>
     <row r="9" spans="1:9" x14ac:dyDescent="0.3">
@@ -5471,7 +5450,7 @@
         <v>C - Koşullu</v>
       </c>
       <c r="I9" t="s">
-        <v>241</v>
+        <v>238</v>
       </c>
     </row>
     <row r="10" spans="1:9" x14ac:dyDescent="0.3">
@@ -5506,7 +5485,7 @@
         <v>C - Koşullu</v>
       </c>
       <c r="I10" t="s">
-        <v>241</v>
+        <v>238</v>
       </c>
     </row>
     <row r="11" spans="1:9" x14ac:dyDescent="0.3">
@@ -5541,7 +5520,7 @@
         <v>C - Koşullu</v>
       </c>
       <c r="I11" t="s">
-        <v>241</v>
+        <v>238</v>
       </c>
     </row>
     <row r="12" spans="1:9" x14ac:dyDescent="0.3">
@@ -5576,7 +5555,7 @@
         <v>D - Zayıf</v>
       </c>
       <c r="I12" t="s">
-        <v>241</v>
+        <v>238</v>
       </c>
     </row>
     <row r="13" spans="1:9" x14ac:dyDescent="0.3">
@@ -5611,7 +5590,7 @@
         <v>C - Koşullu</v>
       </c>
       <c r="I13" t="s">
-        <v>241</v>
+        <v>238</v>
       </c>
     </row>
     <row r="14" spans="1:9" x14ac:dyDescent="0.3">
@@ -5623,11 +5602,11 @@
       </c>
       <c r="C14">
         <f>MIN(100,MAX(0,(Aday_Verileri!P14/700)*55+(Aday_Verileri!G14/10000)*25+(1/(1+Aday_Verileri!R14/800))*20))</f>
-        <v>80.82976708371767</v>
+        <v>59.289871895629915</v>
       </c>
       <c r="D14">
         <f>MIN(100,MAX(0,100-Aday_Verileri!AK14*5))</f>
-        <v>25.786854718075517</v>
+        <v>47.717995075681515</v>
       </c>
       <c r="E14">
         <f>IF(Aday_Verileri!AL14="Yüksek/Orta",80,55)</f>
@@ -5639,14 +5618,14 @@
       </c>
       <c r="G14">
         <f t="shared" si="0"/>
-        <v>55.1073059848135</v>
+        <v>54.167247034740498</v>
       </c>
       <c r="H14" t="str">
         <f t="shared" si="1"/>
         <v>C - Koşullu</v>
       </c>
       <c r="I14" t="s">
-        <v>241</v>
+        <v>238</v>
       </c>
     </row>
     <row r="15" spans="1:9" x14ac:dyDescent="0.3">
@@ -5654,15 +5633,15 @@
         <v>14</v>
       </c>
       <c r="B15" t="s">
-        <v>145</v>
+        <v>144</v>
       </c>
       <c r="C15">
         <f>MIN(100,MAX(0,(Aday_Verileri!P15/700)*55+(Aday_Verileri!G15/10000)*25+(1/(1+Aday_Verileri!R15/800))*20))</f>
-        <v>90.023683093801111</v>
+        <v>67.003600316314476</v>
       </c>
       <c r="D15">
         <f>MIN(100,MAX(0,100-Aday_Verileri!AK15*5))</f>
-        <v>25.786854718075517</v>
+        <v>47.646537403781053</v>
       </c>
       <c r="E15">
         <f>IF(Aday_Verileri!AL15="Yüksek/Orta",80,55)</f>
@@ -5674,14 +5653,14 @@
       </c>
       <c r="G15">
         <f t="shared" si="0"/>
-        <v>60.284872388846878</v>
+        <v>58.727728217849162</v>
       </c>
       <c r="H15" t="str">
         <f t="shared" si="1"/>
         <v>C - Koşullu</v>
       </c>
       <c r="I15" t="s">
-        <v>241</v>
+        <v>238</v>
       </c>
     </row>
     <row r="16" spans="1:9" x14ac:dyDescent="0.3">
@@ -5689,15 +5668,15 @@
         <v>15</v>
       </c>
       <c r="B16" t="s">
-        <v>150</v>
+        <v>148</v>
       </c>
       <c r="C16">
         <f>MIN(100,MAX(0,(Aday_Verileri!P16/700)*55+(Aday_Verileri!G16/10000)*25+(1/(1+Aday_Verileri!R16/800))*20))</f>
-        <v>68.542855280033592</v>
+        <v>90.023683093801111</v>
       </c>
       <c r="D16">
         <f>MIN(100,MAX(0,100-Aday_Verileri!AK16*5))</f>
-        <v>33.871932974266898</v>
+        <v>31.214514463807873</v>
       </c>
       <c r="E16">
         <f>IF(Aday_Verileri!AL16="Yüksek/Orta",80,55)</f>
@@ -5705,18 +5684,18 @@
       </c>
       <c r="F16">
         <f>MAX(0,100-IF(ISNUMBER(SEARCH("deniz",Aday_Verileri!C16)),20,0)-IF(ISNUMBER(SEARCH("jeoloji",Aday_Verileri!AM16)),15,0)-IF(ISNUMBER(SEARCH("izin",Aday_Verileri!AM16)),15,0)-IF(ISNUMBER(SEARCH("su",Aday_Verileri!AM16)),10,0))</f>
-        <v>65</v>
+        <v>55</v>
       </c>
       <c r="G16">
         <f t="shared" si="0"/>
-        <v>54.522318653006849</v>
+        <v>60.684553299853199</v>
       </c>
       <c r="H16" t="str">
         <f t="shared" si="1"/>
         <v>C - Koşullu</v>
       </c>
       <c r="I16" t="s">
-        <v>241</v>
+        <v>238</v>
       </c>
     </row>
   </sheetData>
@@ -5750,63 +5729,63 @@
   <sheetData>
     <row r="1" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A1" s="1" t="s">
-        <v>242</v>
+        <v>239</v>
       </c>
       <c r="B1" s="1" t="s">
-        <v>243</v>
+        <v>240</v>
       </c>
     </row>
     <row r="2" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A2" t="s">
-        <v>244</v>
+        <v>241</v>
       </c>
       <c r="B2" t="s">
-        <v>245</v>
+        <v>242</v>
       </c>
     </row>
     <row r="3" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A3" t="s">
-        <v>246</v>
+        <v>243</v>
       </c>
       <c r="B3" t="s">
-        <v>247</v>
+        <v>244</v>
       </c>
     </row>
     <row r="4" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A4" t="s">
-        <v>248</v>
+        <v>245</v>
       </c>
       <c r="B4" t="s">
-        <v>249</v>
+        <v>246</v>
       </c>
     </row>
     <row r="5" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A5" t="s">
-        <v>250</v>
+        <v>247</v>
       </c>
       <c r="B5" t="s">
-        <v>251</v>
+        <v>248</v>
       </c>
     </row>
     <row r="6" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A6" t="s">
-        <v>252</v>
+        <v>249</v>
       </c>
       <c r="B6" t="s">
-        <v>253</v>
+        <v>250</v>
       </c>
     </row>
     <row r="7" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A7" t="s">
-        <v>254</v>
+        <v>251</v>
       </c>
       <c r="B7" t="s">
-        <v>255</v>
+        <v>252</v>
       </c>
     </row>
     <row r="8" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A8" t="s">
-        <v>256</v>
+        <v>253</v>
       </c>
       <c r="B8" t="s">
         <v>84</v>
@@ -5814,74 +5793,74 @@
     </row>
     <row r="9" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A9" t="s">
-        <v>257</v>
+        <v>254</v>
       </c>
       <c r="B9" t="s">
-        <v>258</v>
+        <v>255</v>
       </c>
     </row>
     <row r="10" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A10" t="s">
-        <v>259</v>
+        <v>256</v>
       </c>
       <c r="B10" t="s">
-        <v>260</v>
+        <v>257</v>
       </c>
     </row>
     <row r="11" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A11" t="s">
-        <v>261</v>
+        <v>258</v>
       </c>
       <c r="B11" t="s">
-        <v>262</v>
+        <v>259</v>
       </c>
     </row>
     <row r="12" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A12" t="s">
-        <v>263</v>
+        <v>260</v>
       </c>
       <c r="B12" t="s">
-        <v>264</v>
+        <v>261</v>
       </c>
     </row>
     <row r="13" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A13" t="s">
-        <v>265</v>
+        <v>262</v>
       </c>
       <c r="B13" t="s">
-        <v>266</v>
+        <v>263</v>
       </c>
     </row>
     <row r="14" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A14" t="s">
-        <v>267</v>
+        <v>264</v>
       </c>
       <c r="B14" t="s">
-        <v>268</v>
+        <v>265</v>
       </c>
     </row>
     <row r="15" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A15" t="s">
-        <v>269</v>
+        <v>266</v>
       </c>
       <c r="B15" t="s">
-        <v>270</v>
+        <v>267</v>
       </c>
     </row>
     <row r="16" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A16" t="s">
-        <v>271</v>
+        <v>268</v>
       </c>
       <c r="B16" t="s">
-        <v>272</v>
+        <v>269</v>
       </c>
     </row>
     <row r="17" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A17" t="s">
-        <v>273</v>
+        <v>270</v>
       </c>
       <c r="B17" t="s">
-        <v>274</v>
+        <v>271</v>
       </c>
     </row>
   </sheetData>

</xml_diff>